<commit_message>
Project 1 Report JPG added
</commit_message>
<xml_diff>
--- a/TabularProject1/Docs and Final Report/Countrywise Customers and Genderwise Employee Report.xlsx
+++ b/TabularProject1/Docs and Final Report/Countrywise Customers and Genderwise Employee Report.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/6447352ca101c75e/Desktop/ssas-learning/TabularProject1/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/6447352ca101c75e/Desktop/ssas-learning/TabularProject1/Docs and Final Report/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="35" documentId="8_{6D4A07C1-369F-4CD0-9BB6-2E1AAA07C673}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{72E22FA8-DB9A-4222-BDCE-4D75BA7E7E07}"/>
+  <xr:revisionPtr revIDLastSave="45" documentId="8_{6D4A07C1-369F-4CD0-9BB6-2E1AAA07C673}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A46B88F0-F3CB-4157-8E07-EF4DA24B87CA}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{233C0D46-9B65-4FAD-B953-5842E0D9B430}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{233C0D46-9B65-4FAD-B953-5842E0D9B430}"/>
   </bookViews>
   <sheets>
     <sheet name="Countrywise Customer Details" sheetId="1" r:id="rId1"/>
@@ -18,8 +18,8 @@
   </sheets>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="166" r:id="rId3"/>
-    <pivotCache cacheId="181" r:id="rId4"/>
+    <pivotCache cacheId="0" r:id="rId3"/>
+    <pivotCache cacheId="1" r:id="rId4"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -149,13 +149,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" pivotButton="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -462,7 +461,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{72EB6309-AE18-45EA-97F2-937999329489}" name="PivotTable3" cacheId="166" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" fieldListSortAscending="1">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{72EB6309-AE18-45EA-97F2-937999329489}" name="PivotTable3" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" fieldListSortAscending="1">
   <location ref="A1:H4" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="8">
     <pivotField axis="axisRow" allDrilled="1" subtotalTop="0" showAll="0" dataSourceSort="1" defaultSubtotal="0" defaultAttributeDrillState="1">
@@ -604,7 +603,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{18BB7065-90A3-44FC-960A-6ECEC2F622ED}" name="PivotTable4" cacheId="181" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" subtotalHiddenItems="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" fieldListSortAscending="1">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{18BB7065-90A3-44FC-960A-6ECEC2F622ED}" name="PivotTable4" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" subtotalHiddenItems="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" fieldListSortAscending="1">
   <location ref="A1:F4" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="6">
     <pivotField axis="axisRow" allDrilled="1" subtotalTop="0" showAll="0" dataSourceSort="1" defaultSubtotal="0" defaultAttributeDrillState="1">
@@ -1035,14 +1034,14 @@
   <dimension ref="A1:H4"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="12.5546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="23.88671875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.5546875" customWidth="1"/>
+    <col min="2" max="2" width="23.88671875" customWidth="1"/>
     <col min="3" max="3" width="23.21875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="14.5546875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="21" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="24.109375" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="17.33203125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.33203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.3">
@@ -1075,25 +1074,25 @@
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="3">
+      <c r="B2">
         <v>2</v>
       </c>
-      <c r="C2" s="3">
+      <c r="C2">
         <v>5</v>
       </c>
-      <c r="D2" s="3">
+      <c r="D2">
         <v>2</v>
       </c>
-      <c r="E2" s="3">
+      <c r="E2">
         <v>4</v>
       </c>
-      <c r="F2" s="3">
+      <c r="F2">
         <v>2</v>
       </c>
-      <c r="G2" s="3">
+      <c r="G2">
         <v>9</v>
       </c>
-      <c r="H2" s="3">
+      <c r="H2">
         <v>850</v>
       </c>
     </row>
@@ -1101,25 +1100,25 @@
       <c r="A3" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="3">
+      <c r="B3">
         <v>3</v>
       </c>
-      <c r="C3" s="3">
+      <c r="C3">
         <v>5</v>
       </c>
-      <c r="D3" s="3">
+      <c r="D3">
         <v>2</v>
       </c>
-      <c r="E3" s="3">
+      <c r="E3">
         <v>6</v>
       </c>
-      <c r="F3" s="3">
+      <c r="F3">
         <v>2</v>
       </c>
-      <c r="G3" s="3">
+      <c r="G3">
         <v>7</v>
       </c>
-      <c r="H3" s="3">
+      <c r="H3">
         <v>1650</v>
       </c>
     </row>
@@ -1127,25 +1126,25 @@
       <c r="A4" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="3">
+      <c r="B4">
         <v>5</v>
       </c>
-      <c r="C4" s="3">
+      <c r="C4">
         <v>5</v>
       </c>
-      <c r="D4" s="3">
+      <c r="D4">
         <v>2</v>
       </c>
-      <c r="E4" s="3">
+      <c r="E4">
         <v>10</v>
       </c>
-      <c r="F4" s="3">
+      <c r="F4">
         <v>4</v>
       </c>
-      <c r="G4" s="3">
+      <c r="G4">
         <v>16</v>
       </c>
-      <c r="H4" s="3">
+      <c r="H4">
         <v>2500</v>
       </c>
     </row>
@@ -1191,19 +1190,19 @@
       <c r="A2" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="B2" s="3">
+      <c r="B2">
         <v>2</v>
       </c>
-      <c r="C2" s="3">
+      <c r="C2">
         <v>55000</v>
       </c>
-      <c r="D2" s="3">
+      <c r="D2">
         <v>65000</v>
       </c>
-      <c r="E2" s="3">
+      <c r="E2">
         <v>75000</v>
       </c>
-      <c r="F2" s="3">
+      <c r="F2">
         <v>130000</v>
       </c>
     </row>
@@ -1211,19 +1210,19 @@
       <c r="A3" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B3" s="3">
+      <c r="B3">
         <v>3</v>
       </c>
-      <c r="C3" s="3">
+      <c r="C3">
         <v>55000</v>
       </c>
-      <c r="D3" s="3">
+      <c r="D3">
         <v>70000</v>
       </c>
-      <c r="E3" s="3">
+      <c r="E3">
         <v>90000</v>
       </c>
-      <c r="F3" s="3">
+      <c r="F3">
         <v>210000</v>
       </c>
     </row>
@@ -1231,19 +1230,19 @@
       <c r="A4" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="3">
+      <c r="B4">
         <v>5</v>
       </c>
-      <c r="C4" s="3">
+      <c r="C4">
         <v>55000</v>
       </c>
-      <c r="D4" s="3">
+      <c r="D4">
         <v>68000</v>
       </c>
-      <c r="E4" s="3">
+      <c r="E4">
         <v>90000</v>
       </c>
-      <c r="F4" s="3">
+      <c r="F4">
         <v>340000</v>
       </c>
     </row>

</xml_diff>